<commit_message>
vault backup: 2026-04-16 06:07:12
</commit_message>
<xml_diff>
--- a/Asus/Contrataciones/Calculadora_Costos_Comercio.xlsx
+++ b/Asus/Contrataciones/Calculadora_Costos_Comercio.xlsx
@@ -9,6 +9,9 @@
   </bookViews>
   <sheets>
     <sheet name="Calculadora" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Mayo 2026" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Junio 2026" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Julio 2026" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -20,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="97">
   <si>
     <t xml:space="preserve">CALCULADORA DE COSTOS - EMPLEADO DE COMERCIO CCT 130/75</t>
   </si>
@@ -248,20 +251,84 @@
   </si>
   <si>
     <t xml:space="preserve">8. Todas las celdas AMARILLAS son editables. El resto se calcula solo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LIQUIDACIÓN DE SUELDO - MAYO 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vendedor B - 48hs - CCT 130/75</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DATOS DEL MES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Salario neto objetivo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Básico Vendedor B (paritarias)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Presentismo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Años de antigüedad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RECIBO DE SUELDO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Importe Bruto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aporte %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deducción</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Neto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Subtotal Remunerativo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Subtotal No Remunerativo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SUELDO BRUTO TOTAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COSTO PARA LA AGENCIA Y FACTURACIÓN AL CLIENTE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contribuciones patronales</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gasto total de la agencia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IVA 21%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LIQUIDACIÓN DE SUELDO - JUNIO 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LIQUIDACIÓN DE SUELDO - JULIO 2026</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="_(\$* #,##0_);_(\$* \(#,##0\);_(\$* \-_);_(@_)"/>
     <numFmt numFmtId="166" formatCode="0.00"/>
     <numFmt numFmtId="167" formatCode="0.0%"/>
     <numFmt numFmtId="168" formatCode="0"/>
+    <numFmt numFmtId="169" formatCode="_(\$* #,##0_);_(\$* \(#,##0\);_(\$* \-_);_(@_)"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -370,6 +437,14 @@
       <family val="0"/>
       <charset val="1"/>
     </font>
+    <font>
+      <i val="true"/>
+      <sz val="11"/>
+      <color rgb="FF666666"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="11">
     <fill>
@@ -381,7 +456,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF2F5496"/>
-        <bgColor rgb="FF666699"/>
+        <bgColor rgb="FF404040"/>
       </patternFill>
     </fill>
     <fill>
@@ -481,11 +556,15 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="72">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -680,6 +759,90 @@
     </xf>
     <xf numFmtId="164" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="7" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="9" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="13" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="13" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="13" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="9" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="9" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="13" fillId="8" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="9" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -739,7 +902,7 @@
       <rgbColor rgb="FFFFCC00"/>
       <rgbColor rgb="FFFF9900"/>
       <rgbColor rgb="FFCC6600"/>
-      <rgbColor rgb="FF666699"/>
+      <rgbColor rgb="FF666666"/>
       <rgbColor rgb="FF969696"/>
       <rgbColor rgb="FF003366"/>
       <rgbColor rgb="FF339966"/>
@@ -938,738 +1101,738 @@
   <dimension ref="B1:I45"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B1" s="1" t="s">
+    <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="3"/>
-      <c r="E4" s="3" t="s">
+      <c r="C4" s="4"/>
+      <c r="E4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
-      <c r="I4" s="3"/>
-    </row>
-    <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="4" t="s">
+      <c r="F4" s="4"/>
+      <c r="G4" s="4"/>
+      <c r="H4" s="4"/>
+      <c r="I4" s="4"/>
+    </row>
+    <row r="5" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B5" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="5" t="n">
+      <c r="C5" s="6" t="n">
         <v>2200000</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="6" t="s">
+    <row r="6" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B6" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="7" t="n">
+      <c r="C6" s="8" t="n">
         <f aca="false">G8+G9+G10+G11+G12+G13+G14+G15+G16+G17+G18+G19</f>
         <v>2693103.58024691</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="E6" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="F6" s="8"/>
-      <c r="G6" s="8"/>
-      <c r="H6" s="8"/>
-      <c r="I6" s="8"/>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E7" s="9" t="s">
+      <c r="F6" s="9"/>
+      <c r="G6" s="9"/>
+      <c r="H6" s="9"/>
+      <c r="I6" s="9"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="E7" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="F7" s="9" t="s">
+      <c r="F7" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="G7" s="9" t="s">
+      <c r="G7" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="H7" s="9" t="s">
+      <c r="H7" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="I7" s="9" t="s">
+      <c r="I7" s="10" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B8" s="8" t="s">
+      <c r="B8" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="8"/>
-      <c r="E8" s="10" t="s">
+      <c r="C8" s="9"/>
+      <c r="E8" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="F8" s="11" t="s">
+      <c r="F8" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="G8" s="12" t="n">
+      <c r="G8" s="13" t="n">
         <f aca="false">C9</f>
         <v>1094044</v>
       </c>
-      <c r="H8" s="13" t="n">
+      <c r="H8" s="14" t="n">
         <f aca="false">C32</f>
         <v>1.57</v>
       </c>
-      <c r="I8" s="12" t="n">
+      <c r="I8" s="13" t="n">
         <f aca="false">G8*H8</f>
         <v>1717649.08</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="4" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B9" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="5" t="n">
+      <c r="C9" s="6" t="n">
         <v>1094044</v>
       </c>
-      <c r="E9" s="10" t="s">
+      <c r="E9" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="F9" s="11" t="s">
+      <c r="F9" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="G9" s="12" t="n">
+      <c r="G9" s="13" t="n">
         <f aca="false">C9*C12</f>
         <v>91133.8652</v>
       </c>
-      <c r="H9" s="13" t="n">
+      <c r="H9" s="14" t="n">
         <f aca="false">C32</f>
         <v>1.57</v>
       </c>
-      <c r="I9" s="12" t="n">
+      <c r="I9" s="13" t="n">
         <f aca="false">G9*H9</f>
         <v>143080.168364</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="4" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B10" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="5" t="n">
+      <c r="C10" s="6" t="n">
         <v>40000</v>
       </c>
-      <c r="E10" s="10" t="s">
+      <c r="E10" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="F10" s="11" t="s">
+      <c r="F10" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="G10" s="12" t="n">
+      <c r="G10" s="13" t="n">
         <f aca="false">C9*C13*C14</f>
         <v>10940.44</v>
       </c>
-      <c r="H10" s="13" t="n">
+      <c r="H10" s="14" t="n">
         <f aca="false">C32</f>
         <v>1.57</v>
       </c>
-      <c r="I10" s="12" t="n">
+      <c r="I10" s="13" t="n">
         <f aca="false">G10*H10</f>
         <v>17176.4908</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="4" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B11" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C11" s="5" t="n">
+      <c r="C11" s="6" t="n">
         <v>60000</v>
       </c>
-      <c r="E11" s="10" t="s">
+      <c r="E11" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="F11" s="11" t="s">
+      <c r="F11" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="G11" s="12" t="n">
+      <c r="G11" s="13" t="n">
         <f aca="false">((C5-(G14+G15+G16+G17+G18+G19)*(1-C22))/(1-C21)-C9*(1+C12+C13*C14))/(1+C12+C13*C14)</f>
         <v>1269235.5941159</v>
       </c>
-      <c r="H11" s="13" t="n">
+      <c r="H11" s="14" t="n">
         <f aca="false">C32</f>
         <v>1.57</v>
       </c>
-      <c r="I11" s="12" t="n">
+      <c r="I11" s="13" t="n">
         <f aca="false">G11*H11</f>
         <v>1992699.88276196</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="4" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B12" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="C12" s="14" t="n">
+      <c r="C12" s="15" t="n">
         <v>0.0833</v>
       </c>
-      <c r="E12" s="10" t="s">
+      <c r="E12" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="F12" s="11" t="s">
+      <c r="F12" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="G12" s="12" t="n">
+      <c r="G12" s="13" t="n">
         <f aca="false">G11*C12</f>
         <v>105727.324989855</v>
       </c>
-      <c r="H12" s="13" t="n">
+      <c r="H12" s="14" t="n">
         <f aca="false">C32</f>
         <v>1.57</v>
       </c>
-      <c r="I12" s="12" t="n">
+      <c r="I12" s="13" t="n">
         <f aca="false">G12*H12</f>
         <v>165991.900234072</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="4" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B13" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="C13" s="15" t="n">
+      <c r="C13" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="E13" s="10" t="s">
+      <c r="E13" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="F13" s="11" t="s">
+      <c r="F13" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="G13" s="12" t="n">
+      <c r="G13" s="13" t="n">
         <f aca="false">G11*C13*C14</f>
         <v>12692.355941159</v>
       </c>
-      <c r="H13" s="13" t="n">
+      <c r="H13" s="14" t="n">
         <f aca="false">C32</f>
         <v>1.57</v>
       </c>
-      <c r="I13" s="12" t="n">
+      <c r="I13" s="13" t="n">
         <f aca="false">G13*H13</f>
         <v>19926.9988276196</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="4" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B14" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="C14" s="14" t="n">
+      <c r="C14" s="15" t="n">
         <v>0.01</v>
       </c>
-      <c r="E14" s="16" t="s">
+      <c r="E14" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="F14" s="17" t="s">
+      <c r="F14" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="G14" s="18" t="n">
+      <c r="G14" s="19" t="n">
         <f aca="false">C10</f>
         <v>40000</v>
       </c>
-      <c r="H14" s="19" t="n">
+      <c r="H14" s="20" t="n">
         <f aca="false">C33</f>
         <v>1.3</v>
       </c>
-      <c r="I14" s="18" t="n">
+      <c r="I14" s="19" t="n">
         <f aca="false">G14*H14</f>
         <v>52000</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E15" s="16" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="E15" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="F15" s="17" t="s">
+      <c r="F15" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="G15" s="18" t="n">
+      <c r="G15" s="19" t="n">
         <f aca="false">C10*C13*C14</f>
         <v>400</v>
       </c>
-      <c r="H15" s="19" t="n">
+      <c r="H15" s="20" t="n">
         <f aca="false">C33</f>
         <v>1.3</v>
       </c>
-      <c r="I15" s="18" t="n">
+      <c r="I15" s="19" t="n">
         <f aca="false">G15*H15</f>
         <v>520</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B16" s="8" t="s">
+      <c r="B16" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="C16" s="8"/>
-      <c r="E16" s="16" t="s">
+      <c r="C16" s="9"/>
+      <c r="E16" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="F16" s="17" t="s">
+      <c r="F16" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="G16" s="18" t="n">
+      <c r="G16" s="19" t="n">
         <f aca="false">C10*C12</f>
         <v>3332</v>
       </c>
-      <c r="H16" s="19" t="n">
+      <c r="H16" s="20" t="n">
         <f aca="false">C33</f>
         <v>1.3</v>
       </c>
-      <c r="I16" s="18" t="n">
+      <c r="I16" s="19" t="n">
         <f aca="false">G16*H16</f>
         <v>4331.6</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="4" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B17" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="C17" s="14" t="n">
+      <c r="C17" s="15" t="n">
         <v>0.11</v>
       </c>
-      <c r="E17" s="16" t="s">
+      <c r="E17" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="F17" s="17" t="s">
+      <c r="F17" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="G17" s="18" t="n">
+      <c r="G17" s="19" t="n">
         <f aca="false">C11</f>
         <v>60000</v>
       </c>
-      <c r="H17" s="19" t="n">
+      <c r="H17" s="20" t="n">
         <f aca="false">C33</f>
         <v>1.3</v>
       </c>
-      <c r="I17" s="18" t="n">
+      <c r="I17" s="19" t="n">
         <f aca="false">G17*H17</f>
         <v>78000</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="4" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B18" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="C18" s="14" t="n">
+      <c r="C18" s="15" t="n">
         <v>0.03</v>
       </c>
-      <c r="E18" s="16" t="s">
+      <c r="E18" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="F18" s="17" t="s">
+      <c r="F18" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="G18" s="18" t="n">
+      <c r="G18" s="19" t="n">
         <f aca="false">C11*C13*C14</f>
         <v>600</v>
       </c>
-      <c r="H18" s="19" t="n">
+      <c r="H18" s="20" t="n">
         <f aca="false">C33</f>
         <v>1.3</v>
       </c>
-      <c r="I18" s="18" t="n">
+      <c r="I18" s="19" t="n">
         <f aca="false">G18*H18</f>
         <v>780</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="4" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B19" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="C19" s="14" t="n">
+      <c r="C19" s="15" t="n">
         <v>0.03</v>
       </c>
-      <c r="E19" s="16" t="s">
+      <c r="E19" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="F19" s="17" t="s">
+      <c r="F19" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="G19" s="18" t="n">
+      <c r="G19" s="19" t="n">
         <f aca="false">C11*C12</f>
         <v>4998</v>
       </c>
-      <c r="H19" s="19" t="n">
+      <c r="H19" s="20" t="n">
         <f aca="false">C33</f>
         <v>1.3</v>
       </c>
-      <c r="I19" s="18" t="n">
+      <c r="I19" s="19" t="n">
         <f aca="false">G19*H19</f>
         <v>6497.4</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="4" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B20" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="C20" s="14" t="n">
+      <c r="C20" s="15" t="n">
         <v>0.02</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B21" s="6" t="s">
+      <c r="B21" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="C21" s="20" t="n">
+      <c r="C21" s="21" t="n">
         <f aca="false">C17+C18+C19+C20</f>
         <v>0.19</v>
       </c>
-      <c r="E21" s="8" t="s">
+      <c r="E21" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="F21" s="8"/>
-      <c r="G21" s="8"/>
-      <c r="H21" s="8"/>
-      <c r="I21" s="8"/>
-    </row>
-    <row r="22" customFormat="false" ht="16.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B22" s="6" t="s">
+      <c r="F21" s="9"/>
+      <c r="G21" s="9"/>
+      <c r="H21" s="9"/>
+      <c r="I21" s="9"/>
+    </row>
+    <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B22" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="C22" s="20" t="n">
+      <c r="C22" s="21" t="n">
         <f aca="false">C20</f>
         <v>0.02</v>
       </c>
-      <c r="E22" s="21" t="s">
+      <c r="E22" s="22" t="s">
         <v>39</v>
       </c>
-      <c r="F22" s="10"/>
-      <c r="G22" s="22" t="n">
+      <c r="F22" s="11"/>
+      <c r="G22" s="23" t="n">
         <f aca="false">(G8+G9+G10+G11+G12+G13)*(1-C21)+(G14+G15+G16+G17+G18+G19)*(1-C22)</f>
         <v>2200000</v>
       </c>
-      <c r="H22" s="23" t="s">
+      <c r="H22" s="24" t="s">
         <v>40</v>
       </c>
-      <c r="I22" s="23"/>
+      <c r="I22" s="24"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="E23" s="24" t="s">
+      <c r="E23" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="F23" s="25"/>
-      <c r="G23" s="26" t="n">
+      <c r="F23" s="26"/>
+      <c r="G23" s="27" t="n">
         <f aca="false">G8+G9+G10+G11+G12+G13+G14+G15+G16+G17+G18+G19</f>
         <v>2693103.58024691</v>
       </c>
-      <c r="H23" s="27" t="s">
+      <c r="H23" s="28" t="s">
         <v>42</v>
       </c>
-      <c r="I23" s="27"/>
+      <c r="I23" s="28"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B24" s="8" t="s">
+      <c r="B24" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="C24" s="8"/>
-      <c r="E24" s="28" t="s">
+      <c r="C24" s="9"/>
+      <c r="E24" s="29" t="s">
         <v>44</v>
       </c>
-      <c r="F24" s="29"/>
-      <c r="G24" s="30" t="n">
+      <c r="F24" s="30"/>
+      <c r="G24" s="31" t="n">
         <f aca="false">(G8+G9+G10+G11+G12+G13)*(1+C28)+(G14+G15+G16+G17+G18+G19)*(1+C29)</f>
         <v>3394002.34691358</v>
       </c>
-      <c r="H24" s="31" t="s">
+      <c r="H24" s="32" t="s">
         <v>45</v>
       </c>
-      <c r="I24" s="31"/>
-    </row>
-    <row r="25" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B25" s="4" t="s">
+      <c r="I24" s="32"/>
+    </row>
+    <row r="25" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B25" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="C25" s="14" t="n">
+      <c r="C25" s="15" t="n">
         <v>0.18</v>
       </c>
-      <c r="E25" s="32" t="s">
+      <c r="E25" s="33" t="s">
         <v>47</v>
       </c>
-      <c r="F25" s="16"/>
-      <c r="G25" s="33" t="n">
+      <c r="F25" s="17"/>
+      <c r="G25" s="34" t="n">
         <f aca="false">(G8+G9+G10+G11+G12+G13)*(C32-1-C28)+(G14+G15+G16+G17+G18+G19)*(C33-1-C29)</f>
         <v>804651.174074074</v>
       </c>
-      <c r="H25" s="34" t="s">
+      <c r="H25" s="35" t="s">
         <v>48</v>
       </c>
-      <c r="I25" s="34"/>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="4" t="s">
+      <c r="I25" s="35"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B26" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="C26" s="14" t="n">
+      <c r="C26" s="15" t="n">
         <v>0.06</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B27" s="4" t="s">
+      <c r="B27" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="C27" s="14" t="n">
+      <c r="C27" s="15" t="n">
         <v>0.03</v>
       </c>
-      <c r="E27" s="6" t="s">
+      <c r="E27" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="F27" s="4"/>
-      <c r="G27" s="35" t="n">
+      <c r="F27" s="5"/>
+      <c r="G27" s="36" t="n">
         <f aca="false">I8+I9+I10+I11+I12+I13+I14+I15+I16+I17+I18+I19</f>
         <v>4198653.52098766</v>
       </c>
-      <c r="H27" s="36" t="s">
+      <c r="H27" s="37" t="s">
         <v>52</v>
       </c>
-      <c r="I27" s="36"/>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B28" s="6" t="s">
+      <c r="I27" s="37"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B28" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="C28" s="37" t="n">
+      <c r="C28" s="38" t="n">
         <f aca="false">C25+C26+C27</f>
         <v>0.27</v>
       </c>
-      <c r="E28" s="4" t="s">
+      <c r="E28" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="F28" s="4"/>
-      <c r="G28" s="38" t="n">
+      <c r="F28" s="5"/>
+      <c r="G28" s="39" t="n">
         <f aca="false">G27*C34</f>
         <v>881717.239407408</v>
       </c>
-      <c r="H28" s="36"/>
-      <c r="I28" s="36"/>
-    </row>
-    <row r="29" customFormat="false" ht="16.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B29" s="6" t="s">
+      <c r="H28" s="37"/>
+      <c r="I28" s="37"/>
+    </row>
+    <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B29" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="C29" s="37" t="n">
+      <c r="C29" s="38" t="n">
         <f aca="false">C27</f>
         <v>0.03</v>
       </c>
-      <c r="E29" s="39" t="s">
+      <c r="E29" s="40" t="s">
         <v>56</v>
       </c>
-      <c r="F29" s="40"/>
-      <c r="G29" s="41" t="n">
+      <c r="F29" s="41"/>
+      <c r="G29" s="42" t="n">
         <f aca="false">G27+G28</f>
         <v>5080370.76039506</v>
       </c>
-      <c r="H29" s="42" t="s">
+      <c r="H29" s="43" t="s">
         <v>57</v>
       </c>
-      <c r="I29" s="42"/>
+      <c r="I29" s="43"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B31" s="8" t="s">
+      <c r="B31" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="C31" s="8"/>
+      <c r="C31" s="9"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B32" s="4" t="s">
+      <c r="B32" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="C32" s="43" t="n">
+      <c r="C32" s="44" t="n">
         <v>1.57</v>
       </c>
-      <c r="E32" s="44" t="s">
+      <c r="E32" s="45" t="s">
         <v>60</v>
       </c>
-      <c r="F32" s="44"/>
-      <c r="G32" s="44"/>
-      <c r="H32" s="44"/>
-      <c r="I32" s="44"/>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="4" t="s">
+      <c r="F32" s="45"/>
+      <c r="G32" s="45"/>
+      <c r="H32" s="45"/>
+      <c r="I32" s="45"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B33" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="C33" s="43" t="n">
+      <c r="C33" s="44" t="n">
         <v>1.3</v>
       </c>
-      <c r="E33" s="36" t="s">
+      <c r="E33" s="37" t="s">
         <v>62</v>
       </c>
-      <c r="G33" s="45" t="n">
+      <c r="G33" s="46" t="n">
         <f aca="false">G24+G25</f>
         <v>4198653.52098765</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B34" s="4" t="s">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B34" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="C34" s="14" t="n">
+      <c r="C34" s="15" t="n">
         <v>0.21</v>
       </c>
-      <c r="E34" s="36" t="s">
+      <c r="E34" s="37" t="s">
         <v>64</v>
       </c>
-      <c r="G34" s="45" t="n">
+      <c r="G34" s="46" t="n">
         <f aca="false">(G8+G9+G10+G11+G12+G13)*(1-C21)+(G14+G15+G16+G17+G18+G19)*(1-C22)</f>
         <v>2200000</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E35" s="36" t="s">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="E35" s="37" t="s">
         <v>65</v>
       </c>
-      <c r="G35" s="46" t="n">
+      <c r="G35" s="47" t="n">
         <f aca="false">1+C28+(C32-1-C28)</f>
         <v>1.57</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B36" s="36" t="s">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B36" s="37" t="s">
         <v>66</v>
       </c>
-      <c r="C36" s="47" t="n">
+      <c r="C36" s="48" t="n">
         <f aca="false">C32-1-C28</f>
         <v>0.3</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B37" s="48" t="s">
+      <c r="B37" s="49" t="s">
         <v>67</v>
       </c>
-      <c r="C37" s="48"/>
-      <c r="D37" s="48"/>
-      <c r="E37" s="48"/>
-      <c r="F37" s="48"/>
-      <c r="G37" s="48"/>
-      <c r="H37" s="48"/>
-      <c r="I37" s="48"/>
+      <c r="C37" s="49"/>
+      <c r="D37" s="49"/>
+      <c r="E37" s="49"/>
+      <c r="F37" s="49"/>
+      <c r="G37" s="49"/>
+      <c r="H37" s="49"/>
+      <c r="I37" s="49"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B38" s="49" t="s">
+      <c r="B38" s="50" t="s">
         <v>68</v>
       </c>
-      <c r="C38" s="49"/>
-      <c r="D38" s="49"/>
-      <c r="E38" s="49"/>
-      <c r="F38" s="49"/>
-      <c r="G38" s="49"/>
-      <c r="H38" s="49"/>
-      <c r="I38" s="49"/>
+      <c r="C38" s="50"/>
+      <c r="D38" s="50"/>
+      <c r="E38" s="50"/>
+      <c r="F38" s="50"/>
+      <c r="G38" s="50"/>
+      <c r="H38" s="50"/>
+      <c r="I38" s="50"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B39" s="49" t="s">
+      <c r="B39" s="50" t="s">
         <v>69</v>
       </c>
-      <c r="C39" s="49"/>
-      <c r="D39" s="49"/>
-      <c r="E39" s="49"/>
-      <c r="F39" s="49"/>
-      <c r="G39" s="49"/>
-      <c r="H39" s="49"/>
-      <c r="I39" s="49"/>
+      <c r="C39" s="50"/>
+      <c r="D39" s="50"/>
+      <c r="E39" s="50"/>
+      <c r="F39" s="50"/>
+      <c r="G39" s="50"/>
+      <c r="H39" s="50"/>
+      <c r="I39" s="50"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B40" s="49" t="s">
+      <c r="B40" s="50" t="s">
         <v>70</v>
       </c>
-      <c r="C40" s="49"/>
-      <c r="D40" s="49"/>
-      <c r="E40" s="49"/>
-      <c r="F40" s="49"/>
-      <c r="G40" s="49"/>
-      <c r="H40" s="49"/>
-      <c r="I40" s="49"/>
+      <c r="C40" s="50"/>
+      <c r="D40" s="50"/>
+      <c r="E40" s="50"/>
+      <c r="F40" s="50"/>
+      <c r="G40" s="50"/>
+      <c r="H40" s="50"/>
+      <c r="I40" s="50"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B41" s="49" t="s">
+      <c r="B41" s="50" t="s">
         <v>71</v>
       </c>
-      <c r="C41" s="49"/>
-      <c r="D41" s="49"/>
-      <c r="E41" s="49"/>
-      <c r="F41" s="49"/>
-      <c r="G41" s="49"/>
-      <c r="H41" s="49"/>
-      <c r="I41" s="49"/>
+      <c r="C41" s="50"/>
+      <c r="D41" s="50"/>
+      <c r="E41" s="50"/>
+      <c r="F41" s="50"/>
+      <c r="G41" s="50"/>
+      <c r="H41" s="50"/>
+      <c r="I41" s="50"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B42" s="49" t="s">
+      <c r="B42" s="50" t="s">
         <v>72</v>
       </c>
-      <c r="C42" s="49"/>
-      <c r="D42" s="49"/>
-      <c r="E42" s="49"/>
-      <c r="F42" s="49"/>
-      <c r="G42" s="49"/>
-      <c r="H42" s="49"/>
-      <c r="I42" s="49"/>
+      <c r="C42" s="50"/>
+      <c r="D42" s="50"/>
+      <c r="E42" s="50"/>
+      <c r="F42" s="50"/>
+      <c r="G42" s="50"/>
+      <c r="H42" s="50"/>
+      <c r="I42" s="50"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B43" s="49" t="s">
+      <c r="B43" s="50" t="s">
         <v>73</v>
       </c>
-      <c r="C43" s="49"/>
-      <c r="D43" s="49"/>
-      <c r="E43" s="49"/>
-      <c r="F43" s="49"/>
-      <c r="G43" s="49"/>
-      <c r="H43" s="49"/>
-      <c r="I43" s="49"/>
+      <c r="C43" s="50"/>
+      <c r="D43" s="50"/>
+      <c r="E43" s="50"/>
+      <c r="F43" s="50"/>
+      <c r="G43" s="50"/>
+      <c r="H43" s="50"/>
+      <c r="I43" s="50"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B44" s="49" t="s">
+      <c r="B44" s="50" t="s">
         <v>74</v>
       </c>
-      <c r="C44" s="49"/>
-      <c r="D44" s="49"/>
-      <c r="E44" s="49"/>
-      <c r="F44" s="49"/>
-      <c r="G44" s="49"/>
-      <c r="H44" s="49"/>
-      <c r="I44" s="49"/>
+      <c r="C44" s="50"/>
+      <c r="D44" s="50"/>
+      <c r="E44" s="50"/>
+      <c r="F44" s="50"/>
+      <c r="G44" s="50"/>
+      <c r="H44" s="50"/>
+      <c r="I44" s="50"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B45" s="49" t="s">
+      <c r="B45" s="50" t="s">
         <v>75</v>
       </c>
-      <c r="C45" s="49"/>
-      <c r="D45" s="49"/>
-      <c r="E45" s="49"/>
-      <c r="F45" s="49"/>
-      <c r="G45" s="49"/>
-      <c r="H45" s="49"/>
-      <c r="I45" s="49"/>
+      <c r="C45" s="50"/>
+      <c r="D45" s="50"/>
+      <c r="E45" s="50"/>
+      <c r="F45" s="50"/>
+      <c r="G45" s="50"/>
+      <c r="H45" s="50"/>
+      <c r="I45" s="50"/>
     </row>
   </sheetData>
   <mergeCells count="27">
@@ -1709,4 +1872,1858 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <tabColor rgb="FFE2EFDA"/>
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="B1:G39"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="18"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B1" s="51" t="s">
+        <v>76</v>
+      </c>
+      <c r="C1" s="51"/>
+      <c r="D1" s="51"/>
+      <c r="E1" s="51"/>
+      <c r="F1" s="51"/>
+      <c r="G1" s="51"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="52" t="s">
+        <v>77</v>
+      </c>
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
+      <c r="E2" s="52"/>
+      <c r="F2" s="52"/>
+      <c r="G2" s="52"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B4" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
+      <c r="G4" s="4"/>
+    </row>
+    <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B5" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="C5" s="53" t="n">
+        <v>2200000</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B6" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="C6" s="53" t="n">
+        <v>1094044</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B7" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="53" t="n">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B8" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" s="53" t="n">
+        <v>60000</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B9" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="C9" s="15" t="n">
+        <v>0.0833</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B10" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="C10" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B11" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C11" s="15" t="n">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B13" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+      <c r="F13" s="4"/>
+      <c r="G13" s="4"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C14" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="D14" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="E14" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="F14" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="G14" s="10" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="C15" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D15" s="54" t="n">
+        <f aca="false">C6</f>
+        <v>1094044</v>
+      </c>
+      <c r="E15" s="55" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="F15" s="54" t="n">
+        <f aca="false">D15*E15</f>
+        <v>207868.36</v>
+      </c>
+      <c r="G15" s="54" t="n">
+        <f aca="false">D15-F15</f>
+        <v>886175.64</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D16" s="54" t="n">
+        <f aca="false">C6*C9</f>
+        <v>91133.8652</v>
+      </c>
+      <c r="E16" s="55" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="F16" s="54" t="n">
+        <f aca="false">D16*E16</f>
+        <v>17315.434388</v>
+      </c>
+      <c r="G16" s="54" t="n">
+        <f aca="false">D16-F16</f>
+        <v>73818.430812</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D17" s="54" t="n">
+        <f aca="false">C6*C10*C11</f>
+        <v>10940.44</v>
+      </c>
+      <c r="E17" s="55" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="F17" s="54" t="n">
+        <f aca="false">D17*E17</f>
+        <v>2078.6836</v>
+      </c>
+      <c r="G17" s="54" t="n">
+        <f aca="false">D17-F17</f>
+        <v>8861.7564</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D18" s="54" t="n">
+        <f aca="false">((C5-(D21+D22+D23+D24+D25+D26)*(1-0.02))/(1-0.19)-C6*(1+C9+C10*C11))/(1+C9+C10*C11)</f>
+        <v>1269235.5941159</v>
+      </c>
+      <c r="E18" s="55" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="F18" s="54" t="n">
+        <f aca="false">D18*E18</f>
+        <v>241154.762882021</v>
+      </c>
+      <c r="G18" s="54" t="n">
+        <f aca="false">D18-F18</f>
+        <v>1028080.83123388</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B19" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D19" s="54" t="n">
+        <f aca="false">D18*C9</f>
+        <v>105727.324989855</v>
+      </c>
+      <c r="E19" s="55" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="F19" s="54" t="n">
+        <f aca="false">D19*E19</f>
+        <v>20088.1917480724</v>
+      </c>
+      <c r="G19" s="54" t="n">
+        <f aca="false">D19-F19</f>
+        <v>85639.1332417821</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B20" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="C20" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D20" s="54" t="n">
+        <f aca="false">D18*C10*C11</f>
+        <v>12692.355941159</v>
+      </c>
+      <c r="E20" s="55" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="F20" s="54" t="n">
+        <f aca="false">D20*E20</f>
+        <v>2411.54762882021</v>
+      </c>
+      <c r="G20" s="54" t="n">
+        <f aca="false">D20-F20</f>
+        <v>10280.8083123388</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B21" s="17" t="s">
+        <v>17</v>
+      </c>
+      <c r="C21" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="D21" s="56" t="n">
+        <f aca="false">C7</f>
+        <v>40000</v>
+      </c>
+      <c r="E21" s="57" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="F21" s="56" t="n">
+        <f aca="false">D21*E21</f>
+        <v>800</v>
+      </c>
+      <c r="G21" s="56" t="n">
+        <f aca="false">D21-F21</f>
+        <v>39200</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B22" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="C22" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="D22" s="56" t="n">
+        <f aca="false">C7*C10*C11</f>
+        <v>400</v>
+      </c>
+      <c r="E22" s="57" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="F22" s="56" t="n">
+        <f aca="false">D22*E22</f>
+        <v>8</v>
+      </c>
+      <c r="G22" s="56" t="n">
+        <f aca="false">D22-F22</f>
+        <v>392</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B23" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="C23" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="D23" s="56" t="n">
+        <f aca="false">C7*C9</f>
+        <v>3332</v>
+      </c>
+      <c r="E23" s="57" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="F23" s="56" t="n">
+        <f aca="false">D23*E23</f>
+        <v>66.64</v>
+      </c>
+      <c r="G23" s="56" t="n">
+        <f aca="false">D23-F23</f>
+        <v>3265.36</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B24" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="C24" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="D24" s="56" t="n">
+        <f aca="false">C8</f>
+        <v>60000</v>
+      </c>
+      <c r="E24" s="57" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="F24" s="56" t="n">
+        <f aca="false">D24*E24</f>
+        <v>1200</v>
+      </c>
+      <c r="G24" s="56" t="n">
+        <f aca="false">D24-F24</f>
+        <v>58800</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B25" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="C25" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="D25" s="56" t="n">
+        <f aca="false">C8*C10*C11</f>
+        <v>600</v>
+      </c>
+      <c r="E25" s="57" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="F25" s="56" t="n">
+        <f aca="false">D25*E25</f>
+        <v>12</v>
+      </c>
+      <c r="G25" s="56" t="n">
+        <f aca="false">D25-F25</f>
+        <v>588</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B26" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="C26" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="D26" s="56" t="n">
+        <f aca="false">C8*C9</f>
+        <v>4998</v>
+      </c>
+      <c r="E26" s="57" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="F26" s="56" t="n">
+        <f aca="false">D26*E26</f>
+        <v>99.96</v>
+      </c>
+      <c r="G26" s="56" t="n">
+        <f aca="false">D26-F26</f>
+        <v>4898.04</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B27" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="C27" s="58" t="s">
+        <v>14</v>
+      </c>
+      <c r="D27" s="59" t="n">
+        <f aca="false">D15+D16+D17+D18+D19+D20</f>
+        <v>2583773.58024691</v>
+      </c>
+      <c r="E27" s="60"/>
+      <c r="F27" s="59" t="n">
+        <f aca="false">D27*0.19</f>
+        <v>490916.980246914</v>
+      </c>
+      <c r="G27" s="59" t="n">
+        <f aca="false">D27-F27</f>
+        <v>2092856.6</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B28" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="C28" s="58" t="s">
+        <v>26</v>
+      </c>
+      <c r="D28" s="59" t="n">
+        <f aca="false">D21+D22+D23+D24+D25+D26</f>
+        <v>109330</v>
+      </c>
+      <c r="E28" s="60"/>
+      <c r="F28" s="59" t="n">
+        <f aca="false">D28*0.02</f>
+        <v>2186.6</v>
+      </c>
+      <c r="G28" s="59" t="n">
+        <f aca="false">D28-F28</f>
+        <v>107143.4</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B29" s="61" t="s">
+        <v>90</v>
+      </c>
+      <c r="C29" s="26"/>
+      <c r="D29" s="62" t="n">
+        <f aca="false">D15+D16+D17+D18+D19+D20+D21+D22+D23+D24+D25+D26</f>
+        <v>2693103.58024691</v>
+      </c>
+      <c r="E29" s="26"/>
+      <c r="F29" s="62" t="n">
+        <f aca="false">(D15+D16+D17+D18+D19+D20)*0.19+(D21+D22+D23+D24+D25+D26)*0.02</f>
+        <v>493103.580246914</v>
+      </c>
+      <c r="G29" s="63" t="n">
+        <f aca="false">D29-F29</f>
+        <v>2200000</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B31" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="C31" s="4"/>
+      <c r="D31" s="4"/>
+      <c r="E31" s="4"/>
+      <c r="F31" s="4"/>
+      <c r="G31" s="4"/>
+    </row>
+    <row r="32" customFormat="false" ht="16.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B32" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="C32" s="22"/>
+      <c r="D32" s="22"/>
+      <c r="E32" s="22"/>
+      <c r="F32" s="64" t="n">
+        <f aca="false">(D15+D16+D17+D18+D19+D20)*(1-0.19)+(D21+D22+D23+D24+D25+D26)*(1-0.02)</f>
+        <v>2200000</v>
+      </c>
+      <c r="G32" s="64"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B33" s="25" t="s">
+        <v>41</v>
+      </c>
+      <c r="C33" s="25"/>
+      <c r="D33" s="25"/>
+      <c r="E33" s="25"/>
+      <c r="F33" s="65" t="n">
+        <f aca="false">D15+D16+D17+D18+D19+D20+D21+D22+D23+D24+D25+D26</f>
+        <v>2693103.58024691</v>
+      </c>
+      <c r="G33" s="65"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B34" s="29" t="s">
+        <v>92</v>
+      </c>
+      <c r="C34" s="29"/>
+      <c r="D34" s="29"/>
+      <c r="E34" s="29"/>
+      <c r="F34" s="66" t="n">
+        <f aca="false">(D15+D16+D17+D18+D19+D20)*0.27+(D21+D22+D23+D24+D25+D26)*0.03</f>
+        <v>700898.766666667</v>
+      </c>
+      <c r="G34" s="66"/>
+    </row>
+    <row r="35" customFormat="false" ht="16.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B35" s="67" t="s">
+        <v>93</v>
+      </c>
+      <c r="C35" s="67"/>
+      <c r="D35" s="67"/>
+      <c r="E35" s="67"/>
+      <c r="F35" s="68" t="n">
+        <f aca="false">(D15+D16+D17+D18+D19+D20)*(1+0.27)+(D21+D22+D23+D24+D25+D26)*(1+0.03)</f>
+        <v>3394002.34691358</v>
+      </c>
+      <c r="G35" s="68"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B36" s="33" t="s">
+        <v>47</v>
+      </c>
+      <c r="C36" s="33"/>
+      <c r="D36" s="33"/>
+      <c r="E36" s="33"/>
+      <c r="F36" s="69" t="n">
+        <f aca="false">(D15+D16+D17+D18+D19+D20)*(1.57-1-0.27)+(D21+D22+D23+D24+D25+D26)*(1.3-1-0.03)</f>
+        <v>804651.174074074</v>
+      </c>
+      <c r="G36" s="69"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B37" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="C37" s="7"/>
+      <c r="D37" s="7"/>
+      <c r="E37" s="7"/>
+      <c r="F37" s="70" t="n">
+        <f aca="false">(D15+D16+D17+D18+D19+D20)*1.57+(D21+D22+D23+D24+D25+D26)*1.3</f>
+        <v>4198653.52098765</v>
+      </c>
+      <c r="G37" s="70"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B38" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C38" s="5"/>
+      <c r="D38" s="5"/>
+      <c r="E38" s="5"/>
+      <c r="F38" s="71" t="n">
+        <f aca="false">((D15+D16+D17+D18+D19+D20)*1.57+(D21+D22+D23+D24+D25+D26)*1.3)*0.21</f>
+        <v>881717.239407407</v>
+      </c>
+      <c r="G38" s="71"/>
+    </row>
+    <row r="39" customFormat="false" ht="16.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B39" s="40" t="s">
+        <v>56</v>
+      </c>
+      <c r="C39" s="40"/>
+      <c r="D39" s="40"/>
+      <c r="E39" s="40"/>
+      <c r="F39" s="63" t="n">
+        <f aca="false">((D15+D16+D17+D18+D19+D20)*1.57+(D21+D22+D23+D24+D25+D26)*1.3)*(1+0.21)</f>
+        <v>5080370.76039506</v>
+      </c>
+      <c r="G39" s="63"/>
+    </row>
+  </sheetData>
+  <mergeCells count="21">
+    <mergeCell ref="B1:G1"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="B4:G4"/>
+    <mergeCell ref="B13:G13"/>
+    <mergeCell ref="B31:G31"/>
+    <mergeCell ref="B32:E32"/>
+    <mergeCell ref="F32:G32"/>
+    <mergeCell ref="B33:E33"/>
+    <mergeCell ref="F33:G33"/>
+    <mergeCell ref="B34:E34"/>
+    <mergeCell ref="F34:G34"/>
+    <mergeCell ref="B35:E35"/>
+    <mergeCell ref="F35:G35"/>
+    <mergeCell ref="B36:E36"/>
+    <mergeCell ref="F36:G36"/>
+    <mergeCell ref="B37:E37"/>
+    <mergeCell ref="F37:G37"/>
+    <mergeCell ref="B38:E38"/>
+    <mergeCell ref="F38:G38"/>
+    <mergeCell ref="B39:E39"/>
+    <mergeCell ref="F39:G39"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <tabColor rgb="FFE2EFDA"/>
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="B1:G39"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="18"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B1" s="51" t="s">
+        <v>95</v>
+      </c>
+      <c r="C1" s="51"/>
+      <c r="D1" s="51"/>
+      <c r="E1" s="51"/>
+      <c r="F1" s="51"/>
+      <c r="G1" s="51"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="52" t="s">
+        <v>77</v>
+      </c>
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
+      <c r="E2" s="52"/>
+      <c r="F2" s="52"/>
+      <c r="G2" s="52"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B4" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
+      <c r="G4" s="4"/>
+    </row>
+    <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B5" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="C5" s="53" t="n">
+        <v>2200000</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B6" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="C6" s="53" t="n">
+        <v>1094044</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B7" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="53" t="n">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B8" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" s="53" t="n">
+        <v>60000</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B9" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="C9" s="15" t="n">
+        <v>0.0833</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B10" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="C10" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B11" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C11" s="15" t="n">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B13" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+      <c r="F13" s="4"/>
+      <c r="G13" s="4"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C14" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="D14" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="E14" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="F14" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="G14" s="10" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="C15" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D15" s="54" t="n">
+        <f aca="false">C6</f>
+        <v>1094044</v>
+      </c>
+      <c r="E15" s="55" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="F15" s="54" t="n">
+        <f aca="false">D15*E15</f>
+        <v>207868.36</v>
+      </c>
+      <c r="G15" s="54" t="n">
+        <f aca="false">D15-F15</f>
+        <v>886175.64</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D16" s="54" t="n">
+        <f aca="false">C6*C9</f>
+        <v>91133.8652</v>
+      </c>
+      <c r="E16" s="55" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="F16" s="54" t="n">
+        <f aca="false">D16*E16</f>
+        <v>17315.434388</v>
+      </c>
+      <c r="G16" s="54" t="n">
+        <f aca="false">D16-F16</f>
+        <v>73818.430812</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D17" s="54" t="n">
+        <f aca="false">C6*C10*C11</f>
+        <v>10940.44</v>
+      </c>
+      <c r="E17" s="55" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="F17" s="54" t="n">
+        <f aca="false">D17*E17</f>
+        <v>2078.6836</v>
+      </c>
+      <c r="G17" s="54" t="n">
+        <f aca="false">D17-F17</f>
+        <v>8861.7564</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D18" s="54" t="n">
+        <f aca="false">((C5-(D21+D22+D23+D24+D25+D26)*(1-0.02))/(1-0.19)-C6*(1+C9+C10*C11))/(1+C9+C10*C11)</f>
+        <v>1269235.5941159</v>
+      </c>
+      <c r="E18" s="55" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="F18" s="54" t="n">
+        <f aca="false">D18*E18</f>
+        <v>241154.762882021</v>
+      </c>
+      <c r="G18" s="54" t="n">
+        <f aca="false">D18-F18</f>
+        <v>1028080.83123388</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B19" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D19" s="54" t="n">
+        <f aca="false">D18*C9</f>
+        <v>105727.324989855</v>
+      </c>
+      <c r="E19" s="55" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="F19" s="54" t="n">
+        <f aca="false">D19*E19</f>
+        <v>20088.1917480724</v>
+      </c>
+      <c r="G19" s="54" t="n">
+        <f aca="false">D19-F19</f>
+        <v>85639.1332417821</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B20" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="C20" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D20" s="54" t="n">
+        <f aca="false">D18*C10*C11</f>
+        <v>12692.355941159</v>
+      </c>
+      <c r="E20" s="55" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="F20" s="54" t="n">
+        <f aca="false">D20*E20</f>
+        <v>2411.54762882021</v>
+      </c>
+      <c r="G20" s="54" t="n">
+        <f aca="false">D20-F20</f>
+        <v>10280.8083123388</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B21" s="17" t="s">
+        <v>17</v>
+      </c>
+      <c r="C21" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="D21" s="56" t="n">
+        <f aca="false">C7</f>
+        <v>40000</v>
+      </c>
+      <c r="E21" s="57" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="F21" s="56" t="n">
+        <f aca="false">D21*E21</f>
+        <v>800</v>
+      </c>
+      <c r="G21" s="56" t="n">
+        <f aca="false">D21-F21</f>
+        <v>39200</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B22" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="C22" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="D22" s="56" t="n">
+        <f aca="false">C7*C10*C11</f>
+        <v>400</v>
+      </c>
+      <c r="E22" s="57" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="F22" s="56" t="n">
+        <f aca="false">D22*E22</f>
+        <v>8</v>
+      </c>
+      <c r="G22" s="56" t="n">
+        <f aca="false">D22-F22</f>
+        <v>392</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B23" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="C23" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="D23" s="56" t="n">
+        <f aca="false">C7*C9</f>
+        <v>3332</v>
+      </c>
+      <c r="E23" s="57" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="F23" s="56" t="n">
+        <f aca="false">D23*E23</f>
+        <v>66.64</v>
+      </c>
+      <c r="G23" s="56" t="n">
+        <f aca="false">D23-F23</f>
+        <v>3265.36</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B24" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="C24" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="D24" s="56" t="n">
+        <f aca="false">C8</f>
+        <v>60000</v>
+      </c>
+      <c r="E24" s="57" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="F24" s="56" t="n">
+        <f aca="false">D24*E24</f>
+        <v>1200</v>
+      </c>
+      <c r="G24" s="56" t="n">
+        <f aca="false">D24-F24</f>
+        <v>58800</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B25" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="C25" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="D25" s="56" t="n">
+        <f aca="false">C8*C10*C11</f>
+        <v>600</v>
+      </c>
+      <c r="E25" s="57" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="F25" s="56" t="n">
+        <f aca="false">D25*E25</f>
+        <v>12</v>
+      </c>
+      <c r="G25" s="56" t="n">
+        <f aca="false">D25-F25</f>
+        <v>588</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B26" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="C26" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="D26" s="56" t="n">
+        <f aca="false">C8*C9</f>
+        <v>4998</v>
+      </c>
+      <c r="E26" s="57" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="F26" s="56" t="n">
+        <f aca="false">D26*E26</f>
+        <v>99.96</v>
+      </c>
+      <c r="G26" s="56" t="n">
+        <f aca="false">D26-F26</f>
+        <v>4898.04</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B27" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="C27" s="58" t="s">
+        <v>14</v>
+      </c>
+      <c r="D27" s="59" t="n">
+        <f aca="false">D15+D16+D17+D18+D19+D20</f>
+        <v>2583773.58024691</v>
+      </c>
+      <c r="E27" s="60"/>
+      <c r="F27" s="59" t="n">
+        <f aca="false">D27*0.19</f>
+        <v>490916.980246914</v>
+      </c>
+      <c r="G27" s="59" t="n">
+        <f aca="false">D27-F27</f>
+        <v>2092856.6</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B28" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="C28" s="58" t="s">
+        <v>26</v>
+      </c>
+      <c r="D28" s="59" t="n">
+        <f aca="false">D21+D22+D23+D24+D25+D26</f>
+        <v>109330</v>
+      </c>
+      <c r="E28" s="60"/>
+      <c r="F28" s="59" t="n">
+        <f aca="false">D28*0.02</f>
+        <v>2186.6</v>
+      </c>
+      <c r="G28" s="59" t="n">
+        <f aca="false">D28-F28</f>
+        <v>107143.4</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B29" s="61" t="s">
+        <v>90</v>
+      </c>
+      <c r="C29" s="26"/>
+      <c r="D29" s="62" t="n">
+        <f aca="false">D15+D16+D17+D18+D19+D20+D21+D22+D23+D24+D25+D26</f>
+        <v>2693103.58024691</v>
+      </c>
+      <c r="E29" s="26"/>
+      <c r="F29" s="62" t="n">
+        <f aca="false">(D15+D16+D17+D18+D19+D20)*0.19+(D21+D22+D23+D24+D25+D26)*0.02</f>
+        <v>493103.580246914</v>
+      </c>
+      <c r="G29" s="63" t="n">
+        <f aca="false">D29-F29</f>
+        <v>2200000</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B31" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="C31" s="4"/>
+      <c r="D31" s="4"/>
+      <c r="E31" s="4"/>
+      <c r="F31" s="4"/>
+      <c r="G31" s="4"/>
+    </row>
+    <row r="32" customFormat="false" ht="16.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B32" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="C32" s="22"/>
+      <c r="D32" s="22"/>
+      <c r="E32" s="22"/>
+      <c r="F32" s="64" t="n">
+        <f aca="false">(D15+D16+D17+D18+D19+D20)*(1-0.19)+(D21+D22+D23+D24+D25+D26)*(1-0.02)</f>
+        <v>2200000</v>
+      </c>
+      <c r="G32" s="64"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B33" s="25" t="s">
+        <v>41</v>
+      </c>
+      <c r="C33" s="25"/>
+      <c r="D33" s="25"/>
+      <c r="E33" s="25"/>
+      <c r="F33" s="65" t="n">
+        <f aca="false">D15+D16+D17+D18+D19+D20+D21+D22+D23+D24+D25+D26</f>
+        <v>2693103.58024691</v>
+      </c>
+      <c r="G33" s="65"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B34" s="29" t="s">
+        <v>92</v>
+      </c>
+      <c r="C34" s="29"/>
+      <c r="D34" s="29"/>
+      <c r="E34" s="29"/>
+      <c r="F34" s="66" t="n">
+        <f aca="false">(D15+D16+D17+D18+D19+D20)*0.27+(D21+D22+D23+D24+D25+D26)*0.03</f>
+        <v>700898.766666667</v>
+      </c>
+      <c r="G34" s="66"/>
+    </row>
+    <row r="35" customFormat="false" ht="16.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B35" s="67" t="s">
+        <v>93</v>
+      </c>
+      <c r="C35" s="67"/>
+      <c r="D35" s="67"/>
+      <c r="E35" s="67"/>
+      <c r="F35" s="68" t="n">
+        <f aca="false">(D15+D16+D17+D18+D19+D20)*(1+0.27)+(D21+D22+D23+D24+D25+D26)*(1+0.03)</f>
+        <v>3394002.34691358</v>
+      </c>
+      <c r="G35" s="68"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B36" s="33" t="s">
+        <v>47</v>
+      </c>
+      <c r="C36" s="33"/>
+      <c r="D36" s="33"/>
+      <c r="E36" s="33"/>
+      <c r="F36" s="69" t="n">
+        <f aca="false">(D15+D16+D17+D18+D19+D20)*(1.57-1-0.27)+(D21+D22+D23+D24+D25+D26)*(1.3-1-0.03)</f>
+        <v>804651.174074074</v>
+      </c>
+      <c r="G36" s="69"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B37" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="C37" s="7"/>
+      <c r="D37" s="7"/>
+      <c r="E37" s="7"/>
+      <c r="F37" s="70" t="n">
+        <f aca="false">(D15+D16+D17+D18+D19+D20)*1.57+(D21+D22+D23+D24+D25+D26)*1.3</f>
+        <v>4198653.52098765</v>
+      </c>
+      <c r="G37" s="70"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B38" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C38" s="5"/>
+      <c r="D38" s="5"/>
+      <c r="E38" s="5"/>
+      <c r="F38" s="71" t="n">
+        <f aca="false">((D15+D16+D17+D18+D19+D20)*1.57+(D21+D22+D23+D24+D25+D26)*1.3)*0.21</f>
+        <v>881717.239407407</v>
+      </c>
+      <c r="G38" s="71"/>
+    </row>
+    <row r="39" customFormat="false" ht="16.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B39" s="40" t="s">
+        <v>56</v>
+      </c>
+      <c r="C39" s="40"/>
+      <c r="D39" s="40"/>
+      <c r="E39" s="40"/>
+      <c r="F39" s="63" t="n">
+        <f aca="false">((D15+D16+D17+D18+D19+D20)*1.57+(D21+D22+D23+D24+D25+D26)*1.3)*(1+0.21)</f>
+        <v>5080370.76039506</v>
+      </c>
+      <c r="G39" s="63"/>
+    </row>
+  </sheetData>
+  <mergeCells count="21">
+    <mergeCell ref="B1:G1"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="B4:G4"/>
+    <mergeCell ref="B13:G13"/>
+    <mergeCell ref="B31:G31"/>
+    <mergeCell ref="B32:E32"/>
+    <mergeCell ref="F32:G32"/>
+    <mergeCell ref="B33:E33"/>
+    <mergeCell ref="F33:G33"/>
+    <mergeCell ref="B34:E34"/>
+    <mergeCell ref="F34:G34"/>
+    <mergeCell ref="B35:E35"/>
+    <mergeCell ref="F35:G35"/>
+    <mergeCell ref="B36:E36"/>
+    <mergeCell ref="F36:G36"/>
+    <mergeCell ref="B37:E37"/>
+    <mergeCell ref="F37:G37"/>
+    <mergeCell ref="B38:E38"/>
+    <mergeCell ref="F38:G38"/>
+    <mergeCell ref="B39:E39"/>
+    <mergeCell ref="F39:G39"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <tabColor rgb="FFE2EFDA"/>
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="B1:G39"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="18"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B1" s="51" t="s">
+        <v>96</v>
+      </c>
+      <c r="C1" s="51"/>
+      <c r="D1" s="51"/>
+      <c r="E1" s="51"/>
+      <c r="F1" s="51"/>
+      <c r="G1" s="51"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="52" t="s">
+        <v>77</v>
+      </c>
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
+      <c r="E2" s="52"/>
+      <c r="F2" s="52"/>
+      <c r="G2" s="52"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B4" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
+      <c r="G4" s="4"/>
+    </row>
+    <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B5" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="C5" s="53" t="n">
+        <v>2200000</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B6" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="C6" s="53" t="n">
+        <v>1094044</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B7" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="53" t="n">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B8" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" s="53" t="n">
+        <v>60000</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B9" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="C9" s="15" t="n">
+        <v>0.0833</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B10" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="C10" s="16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B11" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C11" s="15" t="n">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B13" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+      <c r="F13" s="4"/>
+      <c r="G13" s="4"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C14" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="D14" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="E14" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="F14" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="G14" s="10" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="C15" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D15" s="54" t="n">
+        <f aca="false">C6</f>
+        <v>1094044</v>
+      </c>
+      <c r="E15" s="55" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="F15" s="54" t="n">
+        <f aca="false">D15*E15</f>
+        <v>207868.36</v>
+      </c>
+      <c r="G15" s="54" t="n">
+        <f aca="false">D15-F15</f>
+        <v>886175.64</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D16" s="54" t="n">
+        <f aca="false">C6*C9</f>
+        <v>91133.8652</v>
+      </c>
+      <c r="E16" s="55" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="F16" s="54" t="n">
+        <f aca="false">D16*E16</f>
+        <v>17315.434388</v>
+      </c>
+      <c r="G16" s="54" t="n">
+        <f aca="false">D16-F16</f>
+        <v>73818.430812</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D17" s="54" t="n">
+        <f aca="false">C6*C10*C11</f>
+        <v>10940.44</v>
+      </c>
+      <c r="E17" s="55" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="F17" s="54" t="n">
+        <f aca="false">D17*E17</f>
+        <v>2078.6836</v>
+      </c>
+      <c r="G17" s="54" t="n">
+        <f aca="false">D17-F17</f>
+        <v>8861.7564</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D18" s="54" t="n">
+        <f aca="false">((C5-(D21+D22+D23+D24+D25+D26)*(1-0.02))/(1-0.19)-C6*(1+C9+C10*C11))/(1+C9+C10*C11)</f>
+        <v>1269235.5941159</v>
+      </c>
+      <c r="E18" s="55" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="F18" s="54" t="n">
+        <f aca="false">D18*E18</f>
+        <v>241154.762882021</v>
+      </c>
+      <c r="G18" s="54" t="n">
+        <f aca="false">D18-F18</f>
+        <v>1028080.83123388</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B19" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D19" s="54" t="n">
+        <f aca="false">D18*C9</f>
+        <v>105727.324989855</v>
+      </c>
+      <c r="E19" s="55" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="F19" s="54" t="n">
+        <f aca="false">D19*E19</f>
+        <v>20088.1917480724</v>
+      </c>
+      <c r="G19" s="54" t="n">
+        <f aca="false">D19-F19</f>
+        <v>85639.1332417821</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B20" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="C20" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D20" s="54" t="n">
+        <f aca="false">D18*C10*C11</f>
+        <v>12692.355941159</v>
+      </c>
+      <c r="E20" s="55" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="F20" s="54" t="n">
+        <f aca="false">D20*E20</f>
+        <v>2411.54762882021</v>
+      </c>
+      <c r="G20" s="54" t="n">
+        <f aca="false">D20-F20</f>
+        <v>10280.8083123388</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B21" s="17" t="s">
+        <v>17</v>
+      </c>
+      <c r="C21" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="D21" s="56" t="n">
+        <f aca="false">C7</f>
+        <v>40000</v>
+      </c>
+      <c r="E21" s="57" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="F21" s="56" t="n">
+        <f aca="false">D21*E21</f>
+        <v>800</v>
+      </c>
+      <c r="G21" s="56" t="n">
+        <f aca="false">D21-F21</f>
+        <v>39200</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B22" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="C22" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="D22" s="56" t="n">
+        <f aca="false">C7*C10*C11</f>
+        <v>400</v>
+      </c>
+      <c r="E22" s="57" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="F22" s="56" t="n">
+        <f aca="false">D22*E22</f>
+        <v>8</v>
+      </c>
+      <c r="G22" s="56" t="n">
+        <f aca="false">D22-F22</f>
+        <v>392</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B23" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="C23" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="D23" s="56" t="n">
+        <f aca="false">C7*C9</f>
+        <v>3332</v>
+      </c>
+      <c r="E23" s="57" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="F23" s="56" t="n">
+        <f aca="false">D23*E23</f>
+        <v>66.64</v>
+      </c>
+      <c r="G23" s="56" t="n">
+        <f aca="false">D23-F23</f>
+        <v>3265.36</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B24" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="C24" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="D24" s="56" t="n">
+        <f aca="false">C8</f>
+        <v>60000</v>
+      </c>
+      <c r="E24" s="57" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="F24" s="56" t="n">
+        <f aca="false">D24*E24</f>
+        <v>1200</v>
+      </c>
+      <c r="G24" s="56" t="n">
+        <f aca="false">D24-F24</f>
+        <v>58800</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B25" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="C25" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="D25" s="56" t="n">
+        <f aca="false">C8*C10*C11</f>
+        <v>600</v>
+      </c>
+      <c r="E25" s="57" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="F25" s="56" t="n">
+        <f aca="false">D25*E25</f>
+        <v>12</v>
+      </c>
+      <c r="G25" s="56" t="n">
+        <f aca="false">D25-F25</f>
+        <v>588</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B26" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="C26" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="D26" s="56" t="n">
+        <f aca="false">C8*C9</f>
+        <v>4998</v>
+      </c>
+      <c r="E26" s="57" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="F26" s="56" t="n">
+        <f aca="false">D26*E26</f>
+        <v>99.96</v>
+      </c>
+      <c r="G26" s="56" t="n">
+        <f aca="false">D26-F26</f>
+        <v>4898.04</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B27" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="C27" s="58" t="s">
+        <v>14</v>
+      </c>
+      <c r="D27" s="59" t="n">
+        <f aca="false">D15+D16+D17+D18+D19+D20</f>
+        <v>2583773.58024691</v>
+      </c>
+      <c r="E27" s="60"/>
+      <c r="F27" s="59" t="n">
+        <f aca="false">D27*0.19</f>
+        <v>490916.980246914</v>
+      </c>
+      <c r="G27" s="59" t="n">
+        <f aca="false">D27-F27</f>
+        <v>2092856.6</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B28" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="C28" s="58" t="s">
+        <v>26</v>
+      </c>
+      <c r="D28" s="59" t="n">
+        <f aca="false">D21+D22+D23+D24+D25+D26</f>
+        <v>109330</v>
+      </c>
+      <c r="E28" s="60"/>
+      <c r="F28" s="59" t="n">
+        <f aca="false">D28*0.02</f>
+        <v>2186.6</v>
+      </c>
+      <c r="G28" s="59" t="n">
+        <f aca="false">D28-F28</f>
+        <v>107143.4</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B29" s="61" t="s">
+        <v>90</v>
+      </c>
+      <c r="C29" s="26"/>
+      <c r="D29" s="62" t="n">
+        <f aca="false">D15+D16+D17+D18+D19+D20+D21+D22+D23+D24+D25+D26</f>
+        <v>2693103.58024691</v>
+      </c>
+      <c r="E29" s="26"/>
+      <c r="F29" s="62" t="n">
+        <f aca="false">(D15+D16+D17+D18+D19+D20)*0.19+(D21+D22+D23+D24+D25+D26)*0.02</f>
+        <v>493103.580246914</v>
+      </c>
+      <c r="G29" s="63" t="n">
+        <f aca="false">D29-F29</f>
+        <v>2200000</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B31" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="C31" s="4"/>
+      <c r="D31" s="4"/>
+      <c r="E31" s="4"/>
+      <c r="F31" s="4"/>
+      <c r="G31" s="4"/>
+    </row>
+    <row r="32" customFormat="false" ht="16.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B32" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="C32" s="22"/>
+      <c r="D32" s="22"/>
+      <c r="E32" s="22"/>
+      <c r="F32" s="64" t="n">
+        <f aca="false">(D15+D16+D17+D18+D19+D20)*(1-0.19)+(D21+D22+D23+D24+D25+D26)*(1-0.02)</f>
+        <v>2200000</v>
+      </c>
+      <c r="G32" s="64"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B33" s="25" t="s">
+        <v>41</v>
+      </c>
+      <c r="C33" s="25"/>
+      <c r="D33" s="25"/>
+      <c r="E33" s="25"/>
+      <c r="F33" s="65" t="n">
+        <f aca="false">D15+D16+D17+D18+D19+D20+D21+D22+D23+D24+D25+D26</f>
+        <v>2693103.58024691</v>
+      </c>
+      <c r="G33" s="65"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B34" s="29" t="s">
+        <v>92</v>
+      </c>
+      <c r="C34" s="29"/>
+      <c r="D34" s="29"/>
+      <c r="E34" s="29"/>
+      <c r="F34" s="66" t="n">
+        <f aca="false">(D15+D16+D17+D18+D19+D20)*0.27+(D21+D22+D23+D24+D25+D26)*0.03</f>
+        <v>700898.766666667</v>
+      </c>
+      <c r="G34" s="66"/>
+    </row>
+    <row r="35" customFormat="false" ht="16.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B35" s="67" t="s">
+        <v>93</v>
+      </c>
+      <c r="C35" s="67"/>
+      <c r="D35" s="67"/>
+      <c r="E35" s="67"/>
+      <c r="F35" s="68" t="n">
+        <f aca="false">(D15+D16+D17+D18+D19+D20)*(1+0.27)+(D21+D22+D23+D24+D25+D26)*(1+0.03)</f>
+        <v>3394002.34691358</v>
+      </c>
+      <c r="G35" s="68"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B36" s="33" t="s">
+        <v>47</v>
+      </c>
+      <c r="C36" s="33"/>
+      <c r="D36" s="33"/>
+      <c r="E36" s="33"/>
+      <c r="F36" s="69" t="n">
+        <f aca="false">(D15+D16+D17+D18+D19+D20)*(1.57-1-0.27)+(D21+D22+D23+D24+D25+D26)*(1.3-1-0.03)</f>
+        <v>804651.174074074</v>
+      </c>
+      <c r="G36" s="69"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B37" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="C37" s="7"/>
+      <c r="D37" s="7"/>
+      <c r="E37" s="7"/>
+      <c r="F37" s="70" t="n">
+        <f aca="false">(D15+D16+D17+D18+D19+D20)*1.57+(D21+D22+D23+D24+D25+D26)*1.3</f>
+        <v>4198653.52098765</v>
+      </c>
+      <c r="G37" s="70"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B38" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C38" s="5"/>
+      <c r="D38" s="5"/>
+      <c r="E38" s="5"/>
+      <c r="F38" s="71" t="n">
+        <f aca="false">((D15+D16+D17+D18+D19+D20)*1.57+(D21+D22+D23+D24+D25+D26)*1.3)*0.21</f>
+        <v>881717.239407407</v>
+      </c>
+      <c r="G38" s="71"/>
+    </row>
+    <row r="39" customFormat="false" ht="16.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B39" s="40" t="s">
+        <v>56</v>
+      </c>
+      <c r="C39" s="40"/>
+      <c r="D39" s="40"/>
+      <c r="E39" s="40"/>
+      <c r="F39" s="63" t="n">
+        <f aca="false">((D15+D16+D17+D18+D19+D20)*1.57+(D21+D22+D23+D24+D25+D26)*1.3)*(1+0.21)</f>
+        <v>5080370.76039506</v>
+      </c>
+      <c r="G39" s="63"/>
+    </row>
+  </sheetData>
+  <mergeCells count="21">
+    <mergeCell ref="B1:G1"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="B4:G4"/>
+    <mergeCell ref="B13:G13"/>
+    <mergeCell ref="B31:G31"/>
+    <mergeCell ref="B32:E32"/>
+    <mergeCell ref="F32:G32"/>
+    <mergeCell ref="B33:E33"/>
+    <mergeCell ref="F33:G33"/>
+    <mergeCell ref="B34:E34"/>
+    <mergeCell ref="F34:G34"/>
+    <mergeCell ref="B35:E35"/>
+    <mergeCell ref="F35:G35"/>
+    <mergeCell ref="B36:E36"/>
+    <mergeCell ref="F36:G36"/>
+    <mergeCell ref="B37:E37"/>
+    <mergeCell ref="F37:G37"/>
+    <mergeCell ref="B38:E38"/>
+    <mergeCell ref="F38:G38"/>
+    <mergeCell ref="B39:E39"/>
+    <mergeCell ref="F39:G39"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>